<commit_message>
GBDS MAY FILES 2026 | fliqlo@GBDS
</commit_message>
<xml_diff>
--- a/GBDS MAY FILES 2026/CSR MONTH OF MAY 2026.xlsx
+++ b/GBDS MAY FILES 2026/CSR MONTH OF MAY 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS MAY FILES 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48CCDADE-E7AC-42E2-BB3F-472C4DFF761B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{558776CB-3161-4D13-AB82-6F1A5B799608}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="8" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
   </bookViews>
   <sheets>
     <sheet name="CSR | MAY" sheetId="902" r:id="rId1"/>
@@ -37156,7 +37156,7 @@
       <c r="D36" s="41"/>
       <c r="E36" s="42"/>
       <c r="F36" s="42">
-        <v>902</v>
+        <v>890</v>
       </c>
       <c r="G36" s="42">
         <v>1</v>
@@ -37330,7 +37330,7 @@
       <c r="D42" s="41"/>
       <c r="E42" s="42"/>
       <c r="F42" s="42">
-        <v>902</v>
+        <v>890</v>
       </c>
       <c r="G42" s="42">
         <v>1</v>

</xml_diff>